<commit_message>
Update ekonomikommunikation.xlsx and PRD.md to reflect changes in financial forecasting dynamics. The PRD now includes a detailed analysis of how different scenarios (A, B, C, D) are impacted over time, emphasizing the importance of forward-looking assessments. A new metric for measuring deterioration over the years has been introduced, enhancing the understanding of financial trends and implications.
</commit_message>
<xml_diff>
--- a/ekonomikommunikation/260903/ekonomikommunikation.xlsx
+++ b/ekonomikommunikation/260903/ekonomikommunikation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ekonomi/ekonomikommunikation/260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="143" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3D521BD-34C7-47C1-B2BA-4949A6AD7DA2}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B295B3A-3063-4404-AAB8-781D64E32BCC}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
   </bookViews>
@@ -1879,7 +1879,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB068F04-3376-4E95-B7A8-1B1D55AB1EEB}">
-  <dimension ref="D2:M89"/>
+  <dimension ref="D2:O89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="24.140625" customWidth="1"/>
@@ -2108,7 +2108,7 @@
         <v>-560</v>
       </c>
     </row>
-    <row r="17" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:15" x14ac:dyDescent="0.25">
       <c r="D17" s="4">
         <v>0.22</v>
       </c>
@@ -2136,14 +2136,14 @@
         <v>-1540</v>
       </c>
     </row>
-    <row r="18" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:15" x14ac:dyDescent="0.25">
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F19" t="s">
         <v>14</v>
       </c>
@@ -2163,14 +2163,14 @@
         <v>-500</v>
       </c>
     </row>
-    <row r="20" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:15" x14ac:dyDescent="0.25">
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F21" s="1" t="s">
         <v>15</v>
       </c>
@@ -2196,14 +2196,14 @@
       </c>
       <c r="L21" s="1"/>
     </row>
-    <row r="22" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:15" x14ac:dyDescent="0.25">
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="4:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="F23" s="6" t="s">
         <v>17</v>
       </c>
@@ -2227,32 +2227,37 @@
         <f>K13+K21</f>
         <v>0</v>
       </c>
-      <c r="L23" s="2">
+      <c r="L23" s="2"/>
+      <c r="M23" s="2">
         <f>SUM(G23:K23)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="O23" s="2">
+        <f>M23-fyra_typfall_tid1!M23</f>
+        <v>-1260</v>
+      </c>
+    </row>
+    <row r="24" spans="4:15" x14ac:dyDescent="0.25">
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:15" x14ac:dyDescent="0.25">
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F26" s="1" t="s">
         <v>20</v>
       </c>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:15" x14ac:dyDescent="0.25">
       <c r="G27" s="5" t="s">
         <v>7</v>
       </c>
@@ -2269,7 +2274,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F28" t="s">
         <v>0</v>
       </c>
@@ -2289,7 +2294,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="29" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F29" t="s">
         <v>6</v>
       </c>
@@ -2309,7 +2314,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="30" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
         <v>1</v>
       </c>
@@ -2329,7 +2334,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="31" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F31" t="s">
         <v>2</v>
       </c>
@@ -2345,7 +2350,7 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="4:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:15" x14ac:dyDescent="0.25">
       <c r="F32" t="s">
         <v>3</v>
       </c>
@@ -2359,7 +2364,7 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>
-    <row r="33" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
         <v>4</v>
       </c>
@@ -2369,7 +2374,7 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F34" t="s">
         <v>5</v>
       </c>
@@ -2379,7 +2384,7 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F35" s="1" t="s">
         <v>11</v>
       </c>
@@ -2404,14 +2409,14 @@
         <v>4100</v>
       </c>
     </row>
-    <row r="36" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F37" t="s">
         <v>13</v>
       </c>
@@ -2431,7 +2436,7 @@
         <v>-7000</v>
       </c>
     </row>
-    <row r="38" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F38" t="s">
         <v>16</v>
       </c>
@@ -2451,7 +2456,7 @@
         <v>-560</v>
       </c>
     </row>
-    <row r="39" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F39" t="s">
         <v>18</v>
       </c>
@@ -2476,14 +2481,14 @@
         <v>-1540</v>
       </c>
     </row>
-    <row r="40" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
     </row>
-    <row r="41" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F41" t="s">
         <v>14</v>
       </c>
@@ -2503,14 +2508,14 @@
         <v>-500</v>
       </c>
     </row>
-    <row r="42" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F43" s="1" t="s">
         <v>15</v>
       </c>
@@ -2535,14 +2540,14 @@
         <v>-9600</v>
       </c>
     </row>
-    <row r="44" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
     </row>
-    <row r="45" spans="6:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="6:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="F45" s="6" t="s">
         <v>17</v>
       </c>
@@ -2570,8 +2575,12 @@
         <f>SUM(G45:K45)</f>
         <v>-9500</v>
       </c>
-    </row>
-    <row r="48" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="O45" s="2">
+        <f>M45-fyra_typfall_tid1!M45</f>
+        <v>-6760</v>
+      </c>
+    </row>
+    <row r="48" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F48" s="1" t="s">
         <v>21</v>
       </c>
@@ -2828,7 +2837,7 @@
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
     </row>
-    <row r="65" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F65" s="1" t="s">
         <v>15</v>
       </c>
@@ -2853,14 +2862,14 @@
         <v>-9600</v>
       </c>
     </row>
-    <row r="66" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
     </row>
-    <row r="67" spans="6:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="6:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="F67" t="s">
         <v>17</v>
       </c>
@@ -2888,13 +2897,17 @@
         <f>SUM(G67:K67)</f>
         <v>-16200</v>
       </c>
-    </row>
-    <row r="70" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="O67" s="2">
+        <f>M67-fyra_typfall_tid1!M67</f>
+        <v>-9860</v>
+      </c>
+    </row>
+    <row r="70" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F70" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="71" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G71" s="5" t="s">
         <v>7</v>
       </c>
@@ -2911,7 +2924,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F72" t="s">
         <v>0</v>
       </c>
@@ -2927,7 +2940,7 @@
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
     </row>
-    <row r="73" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F73" t="s">
         <v>6</v>
       </c>
@@ -2941,7 +2954,7 @@
       <c r="J73" s="2"/>
       <c r="K73" s="2"/>
     </row>
-    <row r="74" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F74" t="s">
         <v>1</v>
       </c>
@@ -2953,7 +2966,7 @@
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
     </row>
-    <row r="75" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F75" t="s">
         <v>2</v>
       </c>
@@ -2965,7 +2978,7 @@
       <c r="J75" s="2"/>
       <c r="K75" s="2"/>
     </row>
-    <row r="76" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F76" t="s">
         <v>3</v>
       </c>
@@ -2977,7 +2990,7 @@
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
     </row>
-    <row r="77" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F77" t="s">
         <v>4</v>
       </c>
@@ -2987,7 +3000,7 @@
       <c r="J77" s="2"/>
       <c r="K77" s="2"/>
     </row>
-    <row r="78" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F78" t="s">
         <v>5</v>
       </c>
@@ -2997,7 +3010,7 @@
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
     </row>
-    <row r="79" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F79" s="1" t="s">
         <v>11</v>
       </c>
@@ -3022,14 +3035,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
     </row>
-    <row r="81" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="81" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F81" t="s">
         <v>13</v>
       </c>
@@ -3049,7 +3062,7 @@
         <v>-7000</v>
       </c>
     </row>
-    <row r="82" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F82" t="s">
         <v>16</v>
       </c>
@@ -3069,7 +3082,7 @@
         <v>-560</v>
       </c>
     </row>
-    <row r="83" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F83" t="s">
         <v>18</v>
       </c>
@@ -3094,14 +3107,14 @@
         <v>-1540</v>
       </c>
     </row>
-    <row r="84" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="84" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
       <c r="K84" s="2"/>
     </row>
-    <row r="85" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="85" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F85" t="s">
         <v>14</v>
       </c>
@@ -3121,14 +3134,14 @@
         <v>-500</v>
       </c>
     </row>
-    <row r="86" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
       <c r="K86" s="2"/>
     </row>
-    <row r="87" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="87" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F87" s="1" t="s">
         <v>15</v>
       </c>
@@ -3153,14 +3166,14 @@
         <v>-9600</v>
       </c>
     </row>
-    <row r="88" spans="6:13" x14ac:dyDescent="0.25">
+    <row r="88" spans="6:15" x14ac:dyDescent="0.25">
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
       <c r="K88" s="2"/>
     </row>
-    <row r="89" spans="6:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="6:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="F89" s="6" t="s">
         <v>17</v>
       </c>
@@ -3187,6 +3200,10 @@
       <c r="M89" s="2">
         <f>SUM(G89:K89)</f>
         <v>-28400</v>
+      </c>
+      <c r="O89" s="2">
+        <f>M89-fyra_typfall_tid1!M89</f>
+        <v>-12860</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor Ekonomikommunikation page to feature four groups (AA, BB, CC, DD) instead of a single research group. Update index.html, README.md, and PRD.md to reflect these changes, including new group-specific hover questions and enhanced user interaction elements. Adjust CSS for tooltip functionality and ensure all references are consistent across documentation. This update aims to improve clarity and engagement with the financial forecasting content.
</commit_message>
<xml_diff>
--- a/ekonomikommunikation/260903/ekonomikommunikation.xlsx
+++ b/ekonomikommunikation/260903/ekonomikommunikation.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ekonomi/ekonomikommunikation/260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B295B3A-3063-4404-AAB8-781D64E32BCC}"/>
+  <xr:revisionPtr revIDLastSave="178" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B95A95B-4021-455E-B28A-30E473863085}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
   </bookViews>
   <sheets>
     <sheet name="fyra_typfall_tid1" sheetId="1" r:id="rId1"/>
-    <sheet name="fyra_typfall_tid2" sheetId="2" r:id="rId2"/>
+    <sheet name="fyra_typfall_tid1 (2)" sheetId="3" r:id="rId2"/>
+    <sheet name="fyra_typfall_tid2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="25">
   <si>
     <t>Bidragsgivare 1, VR</t>
   </si>
@@ -1872,12 +1873,1390 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CB101EA-6E48-4161-BC10-21E0771D941E}">
+  <dimension ref="E4:M89"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="24.140625" customWidth="1"/>
+    <col min="7" max="7" width="25.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="G5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1000</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="2">
+        <v>1000</v>
+      </c>
+      <c r="J6" s="2">
+        <v>1000</v>
+      </c>
+      <c r="K6" s="2">
+        <v>1000</v>
+      </c>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H7" s="2">
+        <v>2000</v>
+      </c>
+      <c r="I7" s="2">
+        <v>2000</v>
+      </c>
+      <c r="J7" s="2">
+        <v>2000</v>
+      </c>
+      <c r="K7" s="2">
+        <v>2000</v>
+      </c>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1100</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1100</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1100</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1100</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1100</v>
+      </c>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H9" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I9" s="2">
+        <v>3000</v>
+      </c>
+      <c r="J9" s="2">
+        <v>3000</v>
+      </c>
+      <c r="K9" s="2">
+        <v>3000</v>
+      </c>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="2">
+        <v>500</v>
+      </c>
+      <c r="H10" s="2">
+        <v>400</v>
+      </c>
+      <c r="I10" s="2">
+        <v>700</v>
+      </c>
+      <c r="J10" s="2">
+        <v>900</v>
+      </c>
+      <c r="K10" s="2">
+        <v>1000</v>
+      </c>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11" s="2">
+        <v>700</v>
+      </c>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1800</v>
+      </c>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="3">
+        <f>SUM(G6:G12)</f>
+        <v>10100</v>
+      </c>
+      <c r="H13" s="3">
+        <f>SUM(H6:H12)</f>
+        <v>7500</v>
+      </c>
+      <c r="I13" s="3">
+        <f>SUM(I6:I12)</f>
+        <v>7800</v>
+      </c>
+      <c r="J13" s="3">
+        <f>SUM(J6:J12)</f>
+        <v>8000</v>
+      </c>
+      <c r="K13" s="3">
+        <f>SUM(K6:K12)</f>
+        <v>8100</v>
+      </c>
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="2">
+        <v>-7000</v>
+      </c>
+      <c r="H15" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="I15" s="2">
+        <v>-5150</v>
+      </c>
+      <c r="J15" s="2">
+        <v>-5300</v>
+      </c>
+      <c r="K15" s="2">
+        <v>-5450</v>
+      </c>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="H16" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="I16" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="J16" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="K16" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="E17" s="4">
+        <v>0.22</v>
+      </c>
+      <c r="F17" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="2">
+        <f>0.22*G15</f>
+        <v>-1540</v>
+      </c>
+      <c r="H17" s="2">
+        <f>0.22*H15</f>
+        <v>-1100</v>
+      </c>
+      <c r="I17" s="2">
+        <f>0.22*I15</f>
+        <v>-1133</v>
+      </c>
+      <c r="J17" s="2">
+        <f>0.22*J15</f>
+        <v>-1166</v>
+      </c>
+      <c r="K17" s="2">
+        <f>0.22*K15</f>
+        <v>-1199</v>
+      </c>
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="2">
+        <v>-500</v>
+      </c>
+      <c r="H19" s="2">
+        <v>-500</v>
+      </c>
+      <c r="I19" s="2">
+        <v>-500</v>
+      </c>
+      <c r="J19" s="2">
+        <v>-500</v>
+      </c>
+      <c r="K19" s="2">
+        <v>-500</v>
+      </c>
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="3">
+        <f>SUM(G15:G20)</f>
+        <v>-10040</v>
+      </c>
+      <c r="H21" s="3">
+        <f>SUM(H15:H20)</f>
+        <v>-7600</v>
+      </c>
+      <c r="I21" s="3">
+        <f>SUM(I15:I20)</f>
+        <v>-7783</v>
+      </c>
+      <c r="J21" s="3">
+        <f>SUM(J15:J20)</f>
+        <v>-7966</v>
+      </c>
+      <c r="K21" s="3">
+        <f>SUM(K15:K20)</f>
+        <v>-8149</v>
+      </c>
+      <c r="L21" s="3"/>
+      <c r="M21" s="1"/>
+    </row>
+    <row r="22" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" spans="5:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="7">
+        <f>G13+G21</f>
+        <v>60</v>
+      </c>
+      <c r="H23" s="7">
+        <f>H13+H21</f>
+        <v>-100</v>
+      </c>
+      <c r="I23" s="7">
+        <f>I13+I21</f>
+        <v>17</v>
+      </c>
+      <c r="J23" s="7">
+        <f>J13+J21</f>
+        <v>34</v>
+      </c>
+      <c r="K23" s="7">
+        <f>K13+K21</f>
+        <v>-49</v>
+      </c>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2">
+        <f>SUM(G23:L23)</f>
+        <v>-38</v>
+      </c>
+    </row>
+    <row r="24" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+    </row>
+    <row r="25" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+    </row>
+    <row r="26" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L26" s="2"/>
+    </row>
+    <row r="27" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="G27" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L27" s="2"/>
+    </row>
+    <row r="28" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2">
+        <v>1000</v>
+      </c>
+      <c r="H28" s="2">
+        <v>1000</v>
+      </c>
+      <c r="I28" s="2">
+        <v>1000</v>
+      </c>
+      <c r="J28" s="2">
+        <v>1000</v>
+      </c>
+      <c r="K28" s="2">
+        <v>1000</v>
+      </c>
+      <c r="L28" s="2"/>
+    </row>
+    <row r="29" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F29" t="s">
+        <v>6</v>
+      </c>
+      <c r="G29" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H29" s="2">
+        <v>2000</v>
+      </c>
+      <c r="I29" s="2">
+        <v>2000</v>
+      </c>
+      <c r="J29" s="2">
+        <v>2000</v>
+      </c>
+      <c r="K29" s="2">
+        <v>2000</v>
+      </c>
+      <c r="L29" s="2"/>
+    </row>
+    <row r="30" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F30" t="s">
+        <v>1</v>
+      </c>
+      <c r="G30" s="2">
+        <v>1100</v>
+      </c>
+      <c r="H30" s="2">
+        <v>1100</v>
+      </c>
+      <c r="I30" s="2">
+        <v>1100</v>
+      </c>
+      <c r="J30" s="2">
+        <v>1100</v>
+      </c>
+      <c r="K30" s="2">
+        <v>1100</v>
+      </c>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
+        <v>2</v>
+      </c>
+      <c r="G31" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H31" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I31" s="2">
+        <v>3000</v>
+      </c>
+      <c r="J31" s="2">
+        <v>3000</v>
+      </c>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="F32" t="s">
+        <v>3</v>
+      </c>
+      <c r="G32" s="2">
+        <v>500</v>
+      </c>
+      <c r="H32" s="2">
+        <v>500</v>
+      </c>
+      <c r="I32" s="2">
+        <v>500</v>
+      </c>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+    </row>
+    <row r="33" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F33" t="s">
+        <v>4</v>
+      </c>
+      <c r="G33" s="2">
+        <v>700</v>
+      </c>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+    </row>
+    <row r="34" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F34" t="s">
+        <v>5</v>
+      </c>
+      <c r="G34" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+    </row>
+    <row r="35" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" s="3">
+        <f>SUM(G28:G34)</f>
+        <v>11300</v>
+      </c>
+      <c r="H35" s="3">
+        <f>SUM(H28:H34)</f>
+        <v>7600</v>
+      </c>
+      <c r="I35" s="3">
+        <f>SUM(I28:I34)</f>
+        <v>7600</v>
+      </c>
+      <c r="J35" s="3">
+        <f>SUM(J28:J34)</f>
+        <v>7100</v>
+      </c>
+      <c r="K35" s="3">
+        <f>SUM(K28:K34)</f>
+        <v>4100</v>
+      </c>
+    </row>
+    <row r="36" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+    </row>
+    <row r="37" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F37" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="2">
+        <v>-7000</v>
+      </c>
+      <c r="H37" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="I37" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="J37" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="K37" s="2">
+        <v>-5000</v>
+      </c>
+    </row>
+    <row r="38" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F38" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="H38" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="I38" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="J38" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="K38" s="2">
+        <v>-1000</v>
+      </c>
+    </row>
+    <row r="39" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F39" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="2">
+        <f>0.22*G37</f>
+        <v>-1540</v>
+      </c>
+      <c r="H39" s="2">
+        <f>0.22*H37</f>
+        <v>-1100</v>
+      </c>
+      <c r="I39" s="2">
+        <f>0.22*I37</f>
+        <v>-1100</v>
+      </c>
+      <c r="J39" s="2">
+        <f>0.22*J37</f>
+        <v>-1100</v>
+      </c>
+      <c r="K39" s="2">
+        <f>0.22*K37</f>
+        <v>-1100</v>
+      </c>
+    </row>
+    <row r="40" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+    </row>
+    <row r="41" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" s="2">
+        <v>-500</v>
+      </c>
+      <c r="H41" s="2">
+        <v>-500</v>
+      </c>
+      <c r="I41" s="2">
+        <v>-500</v>
+      </c>
+      <c r="J41" s="2">
+        <v>-500</v>
+      </c>
+      <c r="K41" s="2">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="42" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+    </row>
+    <row r="43" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F43" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G43" s="3">
+        <f>SUM(G37:G42)</f>
+        <v>-10040</v>
+      </c>
+      <c r="H43" s="3">
+        <f>SUM(H37:H42)</f>
+        <v>-7600</v>
+      </c>
+      <c r="I43" s="3">
+        <f>SUM(I37:I42)</f>
+        <v>-7600</v>
+      </c>
+      <c r="J43" s="3">
+        <f>SUM(J37:J42)</f>
+        <v>-7600</v>
+      </c>
+      <c r="K43" s="3">
+        <f>SUM(K37:K42)</f>
+        <v>-7600</v>
+      </c>
+    </row>
+    <row r="44" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+    </row>
+    <row r="45" spans="6:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F45" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G45" s="7">
+        <f>G35+G43</f>
+        <v>1260</v>
+      </c>
+      <c r="H45" s="7">
+        <f>H35+H43</f>
+        <v>0</v>
+      </c>
+      <c r="I45" s="7">
+        <f>I35+I43</f>
+        <v>0</v>
+      </c>
+      <c r="J45" s="7">
+        <f>J35+J43</f>
+        <v>-500</v>
+      </c>
+      <c r="K45" s="7">
+        <f>K35+K43</f>
+        <v>-3500</v>
+      </c>
+      <c r="M45" s="2">
+        <f>SUM(G45:L45)</f>
+        <v>-2740</v>
+      </c>
+    </row>
+    <row r="48" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F48" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="G49" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H49" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K49" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F50" t="s">
+        <v>0</v>
+      </c>
+      <c r="G50" s="2">
+        <v>1000</v>
+      </c>
+      <c r="H50" s="2">
+        <v>1000</v>
+      </c>
+      <c r="I50" s="2">
+        <v>1000</v>
+      </c>
+      <c r="J50" s="2">
+        <v>1000</v>
+      </c>
+      <c r="K50" s="2">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="51" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F51" t="s">
+        <v>6</v>
+      </c>
+      <c r="G51" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H51" s="2">
+        <v>2000</v>
+      </c>
+      <c r="I51" s="2">
+        <v>2000</v>
+      </c>
+      <c r="J51" s="2">
+        <v>2000</v>
+      </c>
+      <c r="K51" s="2">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="52" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F52" t="s">
+        <v>1</v>
+      </c>
+      <c r="G52" s="2">
+        <v>1100</v>
+      </c>
+      <c r="H52" s="2">
+        <v>1100</v>
+      </c>
+      <c r="I52" s="2">
+        <v>1100</v>
+      </c>
+      <c r="J52" s="2">
+        <v>1100</v>
+      </c>
+      <c r="K52" s="2"/>
+    </row>
+    <row r="53" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F53" t="s">
+        <v>2</v>
+      </c>
+      <c r="G53" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H53" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I53" s="2">
+        <v>3000</v>
+      </c>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+    </row>
+    <row r="54" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F54" t="s">
+        <v>3</v>
+      </c>
+      <c r="G54" s="2">
+        <v>500</v>
+      </c>
+      <c r="H54" s="2">
+        <v>500</v>
+      </c>
+      <c r="I54" s="2">
+        <v>500</v>
+      </c>
+      <c r="J54" s="2">
+        <v>500</v>
+      </c>
+      <c r="K54" s="2"/>
+    </row>
+    <row r="55" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F55" t="s">
+        <v>4</v>
+      </c>
+      <c r="G55" s="2">
+        <v>700</v>
+      </c>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
+    </row>
+    <row r="56" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F56" t="s">
+        <v>5</v>
+      </c>
+      <c r="G56" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+      <c r="K56" s="2"/>
+    </row>
+    <row r="57" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F57" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G57" s="3">
+        <f>SUM(G50:G56)</f>
+        <v>11300</v>
+      </c>
+      <c r="H57" s="3">
+        <f>SUM(H50:H56)</f>
+        <v>7600</v>
+      </c>
+      <c r="I57" s="3">
+        <f>SUM(I50:I56)</f>
+        <v>7600</v>
+      </c>
+      <c r="J57" s="3">
+        <f>SUM(J50:J56)</f>
+        <v>4600</v>
+      </c>
+      <c r="K57" s="3">
+        <f>SUM(K50:K56)</f>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="58" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
+      <c r="K58" s="2"/>
+    </row>
+    <row r="59" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F59" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" s="2">
+        <v>-7000</v>
+      </c>
+      <c r="H59" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="I59" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="J59" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="K59" s="2">
+        <v>-5000</v>
+      </c>
+    </row>
+    <row r="60" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F60" t="s">
+        <v>16</v>
+      </c>
+      <c r="G60" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="H60" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="I60" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="J60" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="K60" s="2">
+        <v>-1000</v>
+      </c>
+    </row>
+    <row r="61" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F61" t="s">
+        <v>18</v>
+      </c>
+      <c r="G61" s="2">
+        <f>0.22*G59</f>
+        <v>-1540</v>
+      </c>
+      <c r="H61" s="2">
+        <f>0.22*H59</f>
+        <v>-1100</v>
+      </c>
+      <c r="I61" s="2">
+        <f>0.22*I59</f>
+        <v>-1100</v>
+      </c>
+      <c r="J61" s="2">
+        <f>0.22*J59</f>
+        <v>-1100</v>
+      </c>
+      <c r="K61" s="2">
+        <f>0.22*K59</f>
+        <v>-1100</v>
+      </c>
+    </row>
+    <row r="62" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
+      <c r="I62" s="2"/>
+      <c r="J62" s="2"/>
+      <c r="K62" s="2"/>
+    </row>
+    <row r="63" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F63" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63" s="2">
+        <v>-500</v>
+      </c>
+      <c r="H63" s="2">
+        <v>-500</v>
+      </c>
+      <c r="I63" s="2">
+        <v>-500</v>
+      </c>
+      <c r="J63" s="2">
+        <v>-500</v>
+      </c>
+      <c r="K63" s="2">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="64" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="G64" s="2"/>
+      <c r="H64" s="2"/>
+      <c r="I64" s="2"/>
+      <c r="J64" s="2"/>
+      <c r="K64" s="2"/>
+    </row>
+    <row r="65" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F65" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G65" s="3">
+        <f>SUM(G59:G64)</f>
+        <v>-10040</v>
+      </c>
+      <c r="H65" s="3">
+        <f>SUM(H59:H64)</f>
+        <v>-7600</v>
+      </c>
+      <c r="I65" s="3">
+        <f>SUM(I59:I64)</f>
+        <v>-7600</v>
+      </c>
+      <c r="J65" s="3">
+        <f>SUM(J59:J64)</f>
+        <v>-7600</v>
+      </c>
+      <c r="K65" s="3">
+        <f>SUM(K59:K64)</f>
+        <v>-7600</v>
+      </c>
+    </row>
+    <row r="66" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G66" s="2"/>
+      <c r="H66" s="2"/>
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
+    </row>
+    <row r="67" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F67" t="s">
+        <v>17</v>
+      </c>
+      <c r="G67" s="2">
+        <f>G57+G65</f>
+        <v>1260</v>
+      </c>
+      <c r="H67" s="2">
+        <f>H57+H65</f>
+        <v>0</v>
+      </c>
+      <c r="I67" s="2">
+        <f>I57+I65</f>
+        <v>0</v>
+      </c>
+      <c r="J67" s="2">
+        <f>J57+J65</f>
+        <v>-3000</v>
+      </c>
+      <c r="K67" s="2">
+        <f>K57+K65</f>
+        <v>-4600</v>
+      </c>
+      <c r="M67" s="2">
+        <f>SUM(G67:L67)</f>
+        <v>-6340</v>
+      </c>
+    </row>
+    <row r="70" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F70" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="71" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G71" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H71" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I71" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J71" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K71" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G72" s="2">
+        <v>1000</v>
+      </c>
+      <c r="H72" s="2">
+        <v>1000</v>
+      </c>
+      <c r="I72" s="2">
+        <v>1000</v>
+      </c>
+      <c r="J72" s="2">
+        <v>1000</v>
+      </c>
+      <c r="K72" s="2"/>
+    </row>
+    <row r="73" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F73" t="s">
+        <v>6</v>
+      </c>
+      <c r="G73" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H73" s="2">
+        <v>2000</v>
+      </c>
+      <c r="I73" s="2">
+        <v>2000</v>
+      </c>
+      <c r="J73" s="2">
+        <v>2000</v>
+      </c>
+      <c r="K73" s="2"/>
+    </row>
+    <row r="74" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F74" t="s">
+        <v>1</v>
+      </c>
+      <c r="G74" s="2">
+        <v>1100</v>
+      </c>
+      <c r="H74" s="2">
+        <v>1100</v>
+      </c>
+      <c r="I74" s="2"/>
+      <c r="J74" s="2"/>
+      <c r="K74" s="2"/>
+    </row>
+    <row r="75" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F75" t="s">
+        <v>2</v>
+      </c>
+      <c r="G75" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H75" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I75" s="2"/>
+      <c r="J75" s="2"/>
+      <c r="K75" s="2"/>
+    </row>
+    <row r="76" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F76" t="s">
+        <v>3</v>
+      </c>
+      <c r="G76" s="2">
+        <v>500</v>
+      </c>
+      <c r="H76" s="2">
+        <v>500</v>
+      </c>
+      <c r="I76" s="2"/>
+      <c r="J76" s="2"/>
+      <c r="K76" s="2"/>
+    </row>
+    <row r="77" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F77" t="s">
+        <v>4</v>
+      </c>
+      <c r="G77" s="2">
+        <v>700</v>
+      </c>
+      <c r="H77" s="2"/>
+      <c r="I77" s="2"/>
+      <c r="J77" s="2"/>
+      <c r="K77" s="2"/>
+    </row>
+    <row r="78" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F78" t="s">
+        <v>5</v>
+      </c>
+      <c r="G78" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H78" s="2"/>
+      <c r="I78" s="2"/>
+      <c r="J78" s="2"/>
+      <c r="K78" s="2"/>
+    </row>
+    <row r="79" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F79" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G79" s="3">
+        <f>SUM(G72:G78)</f>
+        <v>11300</v>
+      </c>
+      <c r="H79" s="3">
+        <f>SUM(H72:H78)</f>
+        <v>7600</v>
+      </c>
+      <c r="I79" s="3">
+        <f>SUM(I72:I78)</f>
+        <v>3000</v>
+      </c>
+      <c r="J79" s="3">
+        <f>SUM(J72:J78)</f>
+        <v>3000</v>
+      </c>
+      <c r="K79" s="3">
+        <f>SUM(K72:K78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G80" s="2"/>
+      <c r="H80" s="2"/>
+      <c r="I80" s="2"/>
+      <c r="J80" s="2"/>
+      <c r="K80" s="2"/>
+    </row>
+    <row r="81" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F81" t="s">
+        <v>13</v>
+      </c>
+      <c r="G81" s="2">
+        <v>-7000</v>
+      </c>
+      <c r="H81" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="I81" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="J81" s="2">
+        <v>-5000</v>
+      </c>
+      <c r="K81" s="2">
+        <v>-5000</v>
+      </c>
+    </row>
+    <row r="82" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F82" t="s">
+        <v>16</v>
+      </c>
+      <c r="G82" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="H82" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="I82" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="J82" s="2">
+        <v>-1000</v>
+      </c>
+      <c r="K82" s="2">
+        <v>-1000</v>
+      </c>
+    </row>
+    <row r="83" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F83" t="s">
+        <v>18</v>
+      </c>
+      <c r="G83" s="2">
+        <f>0.22*G81</f>
+        <v>-1540</v>
+      </c>
+      <c r="H83" s="2">
+        <f>0.22*H81</f>
+        <v>-1100</v>
+      </c>
+      <c r="I83" s="2">
+        <f>0.22*I81</f>
+        <v>-1100</v>
+      </c>
+      <c r="J83" s="2">
+        <f>0.22*J81</f>
+        <v>-1100</v>
+      </c>
+      <c r="K83" s="2">
+        <f>0.22*K81</f>
+        <v>-1100</v>
+      </c>
+    </row>
+    <row r="84" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G84" s="2"/>
+      <c r="H84" s="2"/>
+      <c r="I84" s="2"/>
+      <c r="J84" s="2"/>
+      <c r="K84" s="2"/>
+    </row>
+    <row r="85" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F85" t="s">
+        <v>14</v>
+      </c>
+      <c r="G85" s="2">
+        <v>-500</v>
+      </c>
+      <c r="H85" s="2">
+        <v>-500</v>
+      </c>
+      <c r="I85" s="2">
+        <v>-500</v>
+      </c>
+      <c r="J85" s="2">
+        <v>-500</v>
+      </c>
+      <c r="K85" s="2">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="86" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G86" s="2"/>
+      <c r="H86" s="2"/>
+      <c r="I86" s="2"/>
+      <c r="J86" s="2"/>
+      <c r="K86" s="2"/>
+    </row>
+    <row r="87" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F87" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G87" s="3">
+        <f>SUM(G81:G86)</f>
+        <v>-10040</v>
+      </c>
+      <c r="H87" s="3">
+        <f>SUM(H81:H86)</f>
+        <v>-7600</v>
+      </c>
+      <c r="I87" s="3">
+        <f>SUM(I81:I86)</f>
+        <v>-7600</v>
+      </c>
+      <c r="J87" s="3">
+        <f>SUM(J81:J86)</f>
+        <v>-7600</v>
+      </c>
+      <c r="K87" s="3">
+        <f>SUM(K81:K86)</f>
+        <v>-7600</v>
+      </c>
+    </row>
+    <row r="88" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="G88" s="2"/>
+      <c r="H88" s="2"/>
+      <c r="I88" s="2"/>
+      <c r="J88" s="2"/>
+      <c r="K88" s="2"/>
+    </row>
+    <row r="89" spans="6:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F89" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G89" s="7">
+        <f>G79+G87</f>
+        <v>1260</v>
+      </c>
+      <c r="H89" s="7">
+        <f>H79+H87</f>
+        <v>0</v>
+      </c>
+      <c r="I89" s="7">
+        <f>I79+I87</f>
+        <v>-4600</v>
+      </c>
+      <c r="J89" s="7">
+        <f>J79+J87</f>
+        <v>-4600</v>
+      </c>
+      <c r="K89" s="7">
+        <f>K79+K87</f>
+        <v>-7600</v>
+      </c>
+      <c r="M89" s="2">
+        <f>SUM(G89:L89)</f>
+        <v>-15540</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB068F04-3376-4E95-B7A8-1B1D55AB1EEB}">
   <dimension ref="D2:O89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Revise introduction and content structure in index.html for the Ekonomikommunikation page, emphasizing the varying capabilities of groups to secure funding over time. Update PRD.md to reflect changes in messaging and clarify the implications for group dynamics. Correct language errors in process-logg.md while preserving original phrasing. This update aims to enhance clarity and engagement with financial forecasting concepts.
</commit_message>
<xml_diff>
--- a/ekonomikommunikation/260903/ekonomikommunikation.xlsx
+++ b/ekonomikommunikation/260903/ekonomikommunikation.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ekonomi/ekonomikommunikation/260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="178" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B95A95B-4021-455E-B28A-30E473863085}"/>
+  <xr:revisionPtr revIDLastSave="248" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6973DF46-CE82-4476-B9B8-337211596EAF}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
   </bookViews>
   <sheets>
     <sheet name="fyra_typfall_tid1" sheetId="1" r:id="rId1"/>
     <sheet name="fyra_typfall_tid1 (2)" sheetId="3" r:id="rId2"/>
     <sheet name="fyra_typfall_tid2" sheetId="2" r:id="rId3"/>
+    <sheet name="inledning" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="30">
   <si>
     <t>Bidragsgivare 1, VR</t>
   </si>
@@ -112,12 +113,27 @@
   <si>
     <t>X+5</t>
   </si>
+  <si>
+    <t>Jag skulle vilja ändra inledningen, som nu är:</t>
+  </si>
+  <si>
+    <t>Till en inledning som denna, nedanstående text:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Men du får ändra språket, om du anser att du måste, om språket är helt "fel", jag vill dock att du respekterar min stil, </t>
+  </si>
+  <si>
+    <t>Samtidigt är jag medveten att språk, texter, alltid kan förbättras!</t>
+  </si>
+  <si>
+    <t>Jag hoppas du ser, förstår, varför jag vill ändra inledningen, budskapet!</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,6 +171,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -176,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -188,6 +212,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -203,6 +228,302 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="textruta 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A9D956F-E90E-B334-D286-0DA2D6EA7A1D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2962275" y="1343025"/>
+          <a:ext cx="8801100" cy="1304925"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Jag har suttit i samtalet flera gånger. En chef eller ledare vill förlänga en tjänst eller anställa någon ny, och frågar rakt ut om pengarna räcker flera år framåt. Det vanliga svaret är en budget för i år, kanske nästa. Sedan blir hen förvånad över hur lite som egentligen är säkrat därefter.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Den här sidan visar varför förvåningen uppstår, och hur en rapportering som sträcker sig fyra år fram kan motverka den. Här är fyra grupper, AA, BB, CC och DD, som var och en lever på flera tidsbegränsade bidrag samtidigt. Bidragen löper ut ett efter ett. Lönerna gör det inte.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Grupperna skiljer sig åt i två avseenden: hur långt fram de har säkrad finansiering, och hur lätt de har att få in nya intäkter till sin verksamhet. AA har täckning alla år framåt. DD ser tuffast ut. Frågan sidan vill väcka är hur illa det egentligen är för DD, och vad man behöver veta för att avgöra det.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="sv-SE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="textruta 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8DCA596-344F-7725-075B-5CA716A0B459}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3038475" y="3314700"/>
+          <a:ext cx="9010650" cy="2400300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>En chef vill förlänga en tjänst eller anställa någon ny, och frågar rakt ut om pengarna räcker flera år framåt. Det kan vara förvånande att få en sådan fråga. Att jag som ekonom</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> inte lyckats kommunicera hur ekonomini ser ut framåt. Att "nya utgifter" kräver "nya intäkter", nya projektmedel. </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="sv-SE" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Den här sidan visar</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> på fyra olika typfall, fyra olika grupper, som antingen har olika förmåga att i god tid säkra medel framåt, för flera år framåt. Eller kommer vissa grupper, bland annat den grupp vi kallar "DD, få det genuint svårt att få ihop budgeten,  dvs säkra de intäkter som gruppen behöver framgent, för att även i framtiden kunna vara en lika stor grupp. </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:br>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Detta är som sagt fyra olika typer av grupper. Man kan tänka sig att den grupp som tidgare har lätt att säkra intäkter, projektmedel, för flera år framöver, blir en grupp som, av olika anledningar, blir en grupp som har svårt att få in pengar för kommande år. Och tvärtom, en grupp som många år precis, precis, innan deadline har fått in pengar till gruppen, dvs haft mycket dålig framförhållning när det gäller att säkra intäkter för framtiden; av olika anledningar, kanske tur, kanske att deras verksamhet just nu ligger "helt rätt i tiden", så får denna "projektgrupp" mycket "lätt" att säkra inkomster, bidrag, till gruppens löner och övriga utgifter. </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="sv-SE" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="sv-SE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4589,4 +4910,40 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00F3BBD5-3FAA-41EF-B5A8-B504E6CD73DC}">
+  <dimension ref="F2:F30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="6:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F2" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="6:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F12" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="6:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F28" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="6:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F29" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="6:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F30" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance group AA's financial forecasting model in app.js with new cost structures reflecting a 3% annual salary increase and 22% overhead. Update PRD.md and SPEC.md to document these changes, including the introduction of a balance tolerance for minor deviations under 2%. Adjust display logic for "one year later" results to indicate stability for small variations. Ensure all updates align with the project's goal of clearer financial assessments.
</commit_message>
<xml_diff>
--- a/ekonomikommunikation/260903/ekonomikommunikation.xlsx
+++ b/ekonomikommunikation/260903/ekonomikommunikation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ekonomi/ekonomikommunikation/260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6973DF46-CE82-4476-B9B8-337211596EAF}"/>
+  <xr:revisionPtr revIDLastSave="251" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B04493C-D025-490C-8F5E-2A6896C5FEFC}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
   </bookViews>
   <sheets>
     <sheet name="fyra_typfall_tid1" sheetId="1" r:id="rId1"/>
@@ -2202,7 +2202,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CB101EA-6E48-4161-BC10-21E0771D941E}">
-  <dimension ref="E4:M89"/>
+  <dimension ref="D4:M89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="24.140625" customWidth="1"/>
@@ -2438,8 +2438,8 @@
       </c>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E17" s="4">
+    <row r="17" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D17" s="4">
         <v>0.22</v>
       </c>
       <c r="F17" t="s">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:13" x14ac:dyDescent="0.25">
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -2475,7 +2475,7 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F19" t="s">
         <v>14</v>
       </c>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:13" x14ac:dyDescent="0.25">
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -2504,7 +2504,7 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F21" s="1" t="s">
         <v>15</v>
       </c>
@@ -2531,7 +2531,7 @@
       <c r="L21" s="3"/>
       <c r="M21" s="1"/>
     </row>
-    <row r="22" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:13" x14ac:dyDescent="0.25">
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -2539,7 +2539,7 @@
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="5:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="F23" s="6" t="s">
         <v>17</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>-38</v>
       </c>
     </row>
-    <row r="24" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:13" x14ac:dyDescent="0.25">
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -2577,7 +2577,7 @@
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:13" x14ac:dyDescent="0.25">
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
@@ -2585,13 +2585,13 @@
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F26" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:13" x14ac:dyDescent="0.25">
       <c r="G27" s="5" t="s">
         <v>12</v>
       </c>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F28" t="s">
         <v>0</v>
       </c>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F29" t="s">
         <v>6</v>
       </c>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
         <v>1</v>
       </c>
@@ -2672,7 +2672,7 @@
       </c>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F31" t="s">
         <v>2</v>
       </c>
@@ -2691,7 +2691,7 @@
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F32" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Consolidate cost structures for financial forecasting in app.js, applying a 3% annual salary increase and 22% overhead across all groups (AA, BB, CC, DD). Update PRD.md and SPEC.md to reflect these changes, ensuring consistent documentation of financial models. Adjust calculations and results presentation to maintain clarity in financial assessments, including revised "one year later" projections. This update aims to enhance the accuracy and usability of the forecasting tool.
</commit_message>
<xml_diff>
--- a/ekonomikommunikation/260903/ekonomikommunikation.xlsx
+++ b/ekonomikommunikation/260903/ekonomikommunikation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ekonomi/ekonomikommunikation/260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="251" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B04493C-D025-490C-8F5E-2A6896C5FEFC}"/>
+  <xr:revisionPtr revIDLastSave="252" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64138035-B888-4A2C-AC4E-20D93E477F8A}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
   </bookViews>
@@ -3933,8 +3933,8 @@
         <v>0</v>
       </c>
       <c r="O23" s="2">
-        <f>M23-fyra_typfall_tid1!M23</f>
-        <v>-1260</v>
+        <f>M23-'fyra_typfall_tid1 (2)'!M23</f>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="4:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add concluding analysis and ingress to index.html, summarizing the financial outlook for groups AA, BB, CC, and DD. Update PRD.md and SPEC.md to reflect the new content, emphasizing the implications of funding changes and the rullande fyraårsprognos concept. Ensure clarity in the presentation of results and maintain consistency across documentation.
</commit_message>
<xml_diff>
--- a/ekonomikommunikation/260903/ekonomikommunikation.xlsx
+++ b/ekonomikommunikation/260903/ekonomikommunikation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ekonomi/ekonomikommunikation/260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="252" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64138035-B888-4A2C-AC4E-20D93E477F8A}"/>
+  <xr:revisionPtr revIDLastSave="308" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C53F9C82-604B-4C3C-9636-1C63B095C42F}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
   </bookViews>
   <sheets>
     <sheet name="fyra_typfall_tid1" sheetId="1" r:id="rId1"/>
@@ -523,6 +523,81 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="textruta 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{440332CE-EDA0-EC21-B18F-D7501BF7119B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3057525" y="6162675"/>
+          <a:ext cx="9020175" cy="1514475"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100"/>
+            <a:t>Det kan dock noteras att</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1100" baseline="0"/>
+            <a:t> alla grupperna, (AA, BB, CC och DD) har sämre resultat om man tittar över alla de fyra år som prognosen sträcker sig över; ett år framåt (från X+1, till X+5). Grupp AA har 192 tkr sämre resultat, grupp BB har 5492 tkr sämre resultat, grupp CC har 8592 tkr i sämre resultat över alla år, och grupp DD har 11 092 tkr i sämre resultat över alla de fyra år som prognosen stäcker sig. Det måste bero på genuint sämre tider för alla typer av forskargrupper. </a:t>
+          </a:r>
+          <a:endParaRPr lang="sv-SE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2777,13 +2852,13 @@
         <v>-5000</v>
       </c>
       <c r="I37" s="2">
-        <v>-5000</v>
+        <v>-5150</v>
       </c>
       <c r="J37" s="2">
-        <v>-5000</v>
+        <v>-5300</v>
       </c>
       <c r="K37" s="2">
-        <v>-5000</v>
+        <v>-5450</v>
       </c>
     </row>
     <row r="38" spans="6:13" x14ac:dyDescent="0.25">
@@ -2820,15 +2895,15 @@
       </c>
       <c r="I39" s="2">
         <f>0.22*I37</f>
-        <v>-1100</v>
+        <v>-1133</v>
       </c>
       <c r="J39" s="2">
         <f>0.22*J37</f>
-        <v>-1100</v>
+        <v>-1166</v>
       </c>
       <c r="K39" s="2">
         <f>0.22*K37</f>
-        <v>-1100</v>
+        <v>-1199</v>
       </c>
     </row>
     <row r="40" spans="6:13" x14ac:dyDescent="0.25">
@@ -2879,15 +2954,15 @@
       </c>
       <c r="I43" s="3">
         <f>SUM(I37:I42)</f>
-        <v>-7600</v>
+        <v>-7783</v>
       </c>
       <c r="J43" s="3">
         <f>SUM(J37:J42)</f>
-        <v>-7600</v>
+        <v>-7966</v>
       </c>
       <c r="K43" s="3">
         <f>SUM(K37:K42)</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
     </row>
     <row r="44" spans="6:13" x14ac:dyDescent="0.25">
@@ -2911,19 +2986,19 @@
       </c>
       <c r="I45" s="7">
         <f>I35+I43</f>
-        <v>0</v>
+        <v>-183</v>
       </c>
       <c r="J45" s="7">
         <f>J35+J43</f>
-        <v>-500</v>
+        <v>-866</v>
       </c>
       <c r="K45" s="7">
         <f>K35+K43</f>
-        <v>-3500</v>
+        <v>-4049</v>
       </c>
       <c r="M45" s="2">
         <f>SUM(G45:L45)</f>
-        <v>-2740</v>
+        <v>-3838</v>
       </c>
     </row>
     <row r="48" spans="6:13" x14ac:dyDescent="0.25">
@@ -3107,13 +3182,13 @@
         <v>-5000</v>
       </c>
       <c r="I59" s="2">
-        <v>-5000</v>
+        <v>-5150</v>
       </c>
       <c r="J59" s="2">
-        <v>-5000</v>
+        <v>-5300</v>
       </c>
       <c r="K59" s="2">
-        <v>-5000</v>
+        <v>-5450</v>
       </c>
     </row>
     <row r="60" spans="6:11" x14ac:dyDescent="0.25">
@@ -3150,15 +3225,15 @@
       </c>
       <c r="I61" s="2">
         <f>0.22*I59</f>
-        <v>-1100</v>
+        <v>-1133</v>
       </c>
       <c r="J61" s="2">
         <f>0.22*J59</f>
-        <v>-1100</v>
+        <v>-1166</v>
       </c>
       <c r="K61" s="2">
         <f>0.22*K59</f>
-        <v>-1100</v>
+        <v>-1199</v>
       </c>
     </row>
     <row r="62" spans="6:11" x14ac:dyDescent="0.25">
@@ -3209,15 +3284,15 @@
       </c>
       <c r="I65" s="3">
         <f>SUM(I59:I64)</f>
-        <v>-7600</v>
+        <v>-7783</v>
       </c>
       <c r="J65" s="3">
         <f>SUM(J59:J64)</f>
-        <v>-7600</v>
+        <v>-7966</v>
       </c>
       <c r="K65" s="3">
         <f>SUM(K59:K64)</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
     </row>
     <row r="66" spans="6:13" x14ac:dyDescent="0.25">
@@ -3241,19 +3316,19 @@
       </c>
       <c r="I67" s="2">
         <f>I57+I65</f>
-        <v>0</v>
+        <v>-183</v>
       </c>
       <c r="J67" s="2">
         <f>J57+J65</f>
-        <v>-3000</v>
+        <v>-3366</v>
       </c>
       <c r="K67" s="2">
         <f>K57+K65</f>
-        <v>-4600</v>
+        <v>-5149</v>
       </c>
       <c r="M67" s="2">
         <f>SUM(G67:L67)</f>
-        <v>-6340</v>
+        <v>-7438</v>
       </c>
     </row>
     <row r="70" spans="6:13" x14ac:dyDescent="0.25">
@@ -3349,9 +3424,7 @@
       <c r="G76" s="2">
         <v>500</v>
       </c>
-      <c r="H76" s="2">
-        <v>500</v>
-      </c>
+      <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
@@ -3390,7 +3463,7 @@
       </c>
       <c r="H79" s="3">
         <f>SUM(H72:H78)</f>
-        <v>7600</v>
+        <v>7100</v>
       </c>
       <c r="I79" s="3">
         <f>SUM(I72:I78)</f>
@@ -3423,13 +3496,13 @@
         <v>-5000</v>
       </c>
       <c r="I81" s="2">
-        <v>-5000</v>
+        <v>-5150</v>
       </c>
       <c r="J81" s="2">
-        <v>-5000</v>
+        <v>-5300</v>
       </c>
       <c r="K81" s="2">
-        <v>-5000</v>
+        <v>-5450</v>
       </c>
     </row>
     <row r="82" spans="6:13" x14ac:dyDescent="0.25">
@@ -3466,15 +3539,15 @@
       </c>
       <c r="I83" s="2">
         <f>0.22*I81</f>
-        <v>-1100</v>
+        <v>-1133</v>
       </c>
       <c r="J83" s="2">
         <f>0.22*J81</f>
-        <v>-1100</v>
+        <v>-1166</v>
       </c>
       <c r="K83" s="2">
         <f>0.22*K81</f>
-        <v>-1100</v>
+        <v>-1199</v>
       </c>
     </row>
     <row r="84" spans="6:13" x14ac:dyDescent="0.25">
@@ -3525,15 +3598,15 @@
       </c>
       <c r="I87" s="3">
         <f>SUM(I81:I86)</f>
-        <v>-7600</v>
+        <v>-7783</v>
       </c>
       <c r="J87" s="3">
         <f>SUM(J81:J86)</f>
-        <v>-7600</v>
+        <v>-7966</v>
       </c>
       <c r="K87" s="3">
         <f>SUM(K81:K86)</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
     </row>
     <row r="88" spans="6:13" x14ac:dyDescent="0.25">
@@ -3553,23 +3626,23 @@
       </c>
       <c r="H89" s="7">
         <f>H79+H87</f>
-        <v>0</v>
+        <v>-500</v>
       </c>
       <c r="I89" s="7">
         <f>I79+I87</f>
-        <v>-4600</v>
+        <v>-4783</v>
       </c>
       <c r="J89" s="7">
         <f>J79+J87</f>
-        <v>-4600</v>
+        <v>-4966</v>
       </c>
       <c r="K89" s="7">
         <f>K79+K87</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
       <c r="M89" s="2">
         <f>SUM(G89:L89)</f>
-        <v>-15540</v>
+        <v>-17138</v>
       </c>
     </row>
   </sheetData>
@@ -3699,19 +3772,19 @@
         <v>3</v>
       </c>
       <c r="G10" s="2">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="H10" s="2">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="I10" s="2">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="J10" s="2">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="K10" s="2">
-        <v>500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="11" spans="6:11" x14ac:dyDescent="0.25">
@@ -3722,9 +3795,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="2">
-        <v>2000</v>
-      </c>
+      <c r="K11" s="2"/>
     </row>
     <row r="12" spans="6:11" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
@@ -3742,23 +3813,23 @@
       </c>
       <c r="G13" s="3">
         <f>SUM(G6:G12)</f>
-        <v>7600</v>
+        <v>7500</v>
       </c>
       <c r="H13" s="3">
         <f>SUM(H6:H12)</f>
-        <v>7600</v>
+        <v>7800</v>
       </c>
       <c r="I13" s="3">
         <f>SUM(I6:I12)</f>
-        <v>7600</v>
+        <v>8000</v>
       </c>
       <c r="J13" s="3">
         <f>SUM(J6:J12)</f>
-        <v>7600</v>
+        <v>8100</v>
       </c>
       <c r="K13" s="3">
         <f>SUM(K6:K12)</f>
-        <v>9600</v>
+        <v>8200</v>
       </c>
     </row>
     <row r="14" spans="6:11" x14ac:dyDescent="0.25">
@@ -3776,16 +3847,16 @@
         <v>-5000</v>
       </c>
       <c r="H15" s="2">
-        <v>-5000</v>
+        <v>-5150</v>
       </c>
       <c r="I15" s="2">
-        <v>-5000</v>
+        <v>-5300</v>
       </c>
       <c r="J15" s="2">
-        <v>-5000</v>
+        <v>-5450</v>
       </c>
       <c r="K15" s="2">
-        <v>-7000</v>
+        <v>-5600</v>
       </c>
     </row>
     <row r="16" spans="6:11" x14ac:dyDescent="0.25">
@@ -3805,7 +3876,7 @@
         <v>-1000</v>
       </c>
       <c r="K16" s="2">
-        <v>-560</v>
+        <v>-1000</v>
       </c>
     </row>
     <row r="17" spans="4:15" x14ac:dyDescent="0.25">
@@ -3821,19 +3892,19 @@
       </c>
       <c r="H17" s="2">
         <f>0.22*H15</f>
-        <v>-1100</v>
+        <v>-1133</v>
       </c>
       <c r="I17" s="2">
         <f>0.22*I15</f>
-        <v>-1100</v>
+        <v>-1166</v>
       </c>
       <c r="J17" s="2">
         <f>0.22*J15</f>
-        <v>-1100</v>
+        <v>-1199</v>
       </c>
       <c r="K17" s="2">
         <f>0.22*K15</f>
-        <v>-1540</v>
+        <v>-1232</v>
       </c>
     </row>
     <row r="18" spans="4:15" x14ac:dyDescent="0.25">
@@ -3880,19 +3951,19 @@
       </c>
       <c r="H21" s="3">
         <f>SUM(H15:H20)</f>
-        <v>-7600</v>
+        <v>-7783</v>
       </c>
       <c r="I21" s="3">
         <f>SUM(I15:I20)</f>
-        <v>-7600</v>
+        <v>-7966</v>
       </c>
       <c r="J21" s="3">
         <f>SUM(J15:J20)</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
       <c r="K21" s="3">
         <f>SUM(K15:K20)</f>
-        <v>-9600</v>
+        <v>-8332</v>
       </c>
       <c r="L21" s="1"/>
     </row>
@@ -3909,32 +3980,32 @@
       </c>
       <c r="G23" s="7">
         <f>G13+G21</f>
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="H23" s="7">
         <f>H13+H21</f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I23" s="7">
         <f>I13+I21</f>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="J23" s="7">
         <f>J13+J21</f>
-        <v>0</v>
+        <v>-49</v>
       </c>
       <c r="K23" s="7">
         <f>K13+K21</f>
-        <v>0</v>
+        <v>-132</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2">
         <f>SUM(G23:K23)</f>
-        <v>0</v>
+        <v>-230</v>
       </c>
       <c r="O23" s="2">
         <f>M23-'fyra_typfall_tid1 (2)'!M23</f>
-        <v>38</v>
+        <v>-192</v>
       </c>
     </row>
     <row r="24" spans="4:15" x14ac:dyDescent="0.25">
@@ -4124,16 +4195,16 @@
         <v>-5000</v>
       </c>
       <c r="H37" s="2">
-        <v>-5000</v>
+        <v>-5150</v>
       </c>
       <c r="I37" s="2">
-        <v>-5000</v>
+        <v>-5300</v>
       </c>
       <c r="J37" s="2">
-        <v>-5000</v>
+        <v>-5450</v>
       </c>
       <c r="K37" s="2">
-        <v>-7000</v>
+        <v>-5600</v>
       </c>
     </row>
     <row r="38" spans="6:15" x14ac:dyDescent="0.25">
@@ -4153,7 +4224,7 @@
         <v>-1000</v>
       </c>
       <c r="K38" s="2">
-        <v>-560</v>
+        <v>-1000</v>
       </c>
     </row>
     <row r="39" spans="6:15" x14ac:dyDescent="0.25">
@@ -4166,19 +4237,19 @@
       </c>
       <c r="H39" s="2">
         <f>0.22*H37</f>
-        <v>-1100</v>
+        <v>-1133</v>
       </c>
       <c r="I39" s="2">
         <f>0.22*I37</f>
-        <v>-1100</v>
+        <v>-1166</v>
       </c>
       <c r="J39" s="2">
         <f>0.22*J37</f>
-        <v>-1100</v>
+        <v>-1199</v>
       </c>
       <c r="K39" s="2">
         <f>0.22*K37</f>
-        <v>-1540</v>
+        <v>-1232</v>
       </c>
     </row>
     <row r="40" spans="6:15" x14ac:dyDescent="0.25">
@@ -4225,19 +4296,19 @@
       </c>
       <c r="H43" s="3">
         <f>SUM(H37:H42)</f>
-        <v>-7600</v>
+        <v>-7783</v>
       </c>
       <c r="I43" s="3">
         <f>SUM(I37:I42)</f>
-        <v>-7600</v>
+        <v>-7966</v>
       </c>
       <c r="J43" s="3">
         <f>SUM(J37:J42)</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
       <c r="K43" s="3">
         <f>SUM(K37:K42)</f>
-        <v>-9600</v>
+        <v>-8332</v>
       </c>
     </row>
     <row r="44" spans="6:15" x14ac:dyDescent="0.25">
@@ -4257,27 +4328,27 @@
       </c>
       <c r="H45" s="7">
         <f>H35+H43</f>
-        <v>0</v>
+        <v>-183</v>
       </c>
       <c r="I45" s="7">
         <f>I35+I43</f>
-        <v>-500</v>
+        <v>-866</v>
       </c>
       <c r="J45" s="7">
         <f>J35+J43</f>
-        <v>-3500</v>
+        <v>-4049</v>
       </c>
       <c r="K45" s="7">
         <f>K35+K43</f>
-        <v>-5500</v>
+        <v>-4232</v>
       </c>
       <c r="M45" s="2">
         <f>SUM(G45:K45)</f>
-        <v>-9500</v>
+        <v>-9330</v>
       </c>
       <c r="O45" s="2">
-        <f>M45-fyra_typfall_tid1!M45</f>
-        <v>-6760</v>
+        <f>M45-'fyra_typfall_tid1 (2)'!M45</f>
+        <v>-5492</v>
       </c>
     </row>
     <row r="48" spans="6:15" x14ac:dyDescent="0.25">
@@ -4446,16 +4517,16 @@
         <v>-5000</v>
       </c>
       <c r="H59" s="2">
-        <v>-5000</v>
+        <v>-5150</v>
       </c>
       <c r="I59" s="2">
-        <v>-5000</v>
+        <v>-5300</v>
       </c>
       <c r="J59" s="2">
-        <v>-5000</v>
+        <v>-5450</v>
       </c>
       <c r="K59" s="2">
-        <v>-7000</v>
+        <v>-5600</v>
       </c>
     </row>
     <row r="60" spans="6:11" x14ac:dyDescent="0.25">
@@ -4475,7 +4546,7 @@
         <v>-1000</v>
       </c>
       <c r="K60" s="2">
-        <v>-560</v>
+        <v>-1000</v>
       </c>
     </row>
     <row r="61" spans="6:11" x14ac:dyDescent="0.25">
@@ -4488,19 +4559,19 @@
       </c>
       <c r="H61" s="2">
         <f>0.22*H59</f>
-        <v>-1100</v>
+        <v>-1133</v>
       </c>
       <c r="I61" s="2">
         <f>0.22*I59</f>
-        <v>-1100</v>
+        <v>-1166</v>
       </c>
       <c r="J61" s="2">
         <f>0.22*J59</f>
-        <v>-1100</v>
+        <v>-1199</v>
       </c>
       <c r="K61" s="2">
         <f>0.22*K59</f>
-        <v>-1540</v>
+        <v>-1232</v>
       </c>
     </row>
     <row r="62" spans="6:11" x14ac:dyDescent="0.25">
@@ -4547,19 +4618,19 @@
       </c>
       <c r="H65" s="3">
         <f>SUM(H59:H64)</f>
-        <v>-7600</v>
+        <v>-7783</v>
       </c>
       <c r="I65" s="3">
         <f>SUM(I59:I64)</f>
-        <v>-7600</v>
+        <v>-7966</v>
       </c>
       <c r="J65" s="3">
         <f>SUM(J59:J64)</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
       <c r="K65" s="3">
         <f>SUM(K59:K64)</f>
-        <v>-9600</v>
+        <v>-8332</v>
       </c>
     </row>
     <row r="66" spans="6:15" x14ac:dyDescent="0.25">
@@ -4579,27 +4650,27 @@
       </c>
       <c r="H67" s="7">
         <f>H57+H65</f>
-        <v>0</v>
+        <v>-183</v>
       </c>
       <c r="I67" s="7">
         <f>I57+I65</f>
-        <v>-3000</v>
+        <v>-3366</v>
       </c>
       <c r="J67" s="7">
         <f>J57+J65</f>
-        <v>-6600</v>
+        <v>-7149</v>
       </c>
       <c r="K67" s="7">
         <f>K57+K65</f>
-        <v>-6600</v>
+        <v>-5332</v>
       </c>
       <c r="M67" s="2">
         <f>SUM(G67:K67)</f>
-        <v>-16200</v>
+        <v>-16030</v>
       </c>
       <c r="O67" s="2">
-        <f>M67-fyra_typfall_tid1!M67</f>
-        <v>-9860</v>
+        <f>M67-'fyra_typfall_tid1 (2)'!M67</f>
+        <v>-8592</v>
       </c>
     </row>
     <row r="70" spans="6:15" x14ac:dyDescent="0.25">
@@ -4750,16 +4821,16 @@
         <v>-5000</v>
       </c>
       <c r="H81" s="2">
-        <v>-5000</v>
+        <v>-5150</v>
       </c>
       <c r="I81" s="2">
-        <v>-5000</v>
+        <v>-5300</v>
       </c>
       <c r="J81" s="2">
-        <v>-5000</v>
+        <v>-5450</v>
       </c>
       <c r="K81" s="2">
-        <v>-7000</v>
+        <v>-5600</v>
       </c>
     </row>
     <row r="82" spans="6:15" x14ac:dyDescent="0.25">
@@ -4779,7 +4850,7 @@
         <v>-1000</v>
       </c>
       <c r="K82" s="2">
-        <v>-560</v>
+        <v>-1000</v>
       </c>
     </row>
     <row r="83" spans="6:15" x14ac:dyDescent="0.25">
@@ -4792,19 +4863,19 @@
       </c>
       <c r="H83" s="2">
         <f>0.22*H81</f>
-        <v>-1100</v>
+        <v>-1133</v>
       </c>
       <c r="I83" s="2">
         <f>0.22*I81</f>
-        <v>-1100</v>
+        <v>-1166</v>
       </c>
       <c r="J83" s="2">
         <f>0.22*J81</f>
-        <v>-1100</v>
+        <v>-1199</v>
       </c>
       <c r="K83" s="2">
         <f>0.22*K81</f>
-        <v>-1540</v>
+        <v>-1232</v>
       </c>
     </row>
     <row r="84" spans="6:15" x14ac:dyDescent="0.25">
@@ -4851,19 +4922,19 @@
       </c>
       <c r="H87" s="3">
         <f>SUM(H81:H86)</f>
-        <v>-7600</v>
+        <v>-7783</v>
       </c>
       <c r="I87" s="3">
         <f>SUM(I81:I86)</f>
-        <v>-7600</v>
+        <v>-7966</v>
       </c>
       <c r="J87" s="3">
         <f>SUM(J81:J86)</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
       <c r="K87" s="3">
         <f>SUM(K81:K86)</f>
-        <v>-9600</v>
+        <v>-8332</v>
       </c>
     </row>
     <row r="88" spans="6:15" x14ac:dyDescent="0.25">
@@ -4883,27 +4954,27 @@
       </c>
       <c r="H89" s="7">
         <f>H79+H87</f>
-        <v>-4600</v>
+        <v>-4783</v>
       </c>
       <c r="I89" s="7">
         <f>I79+I87</f>
-        <v>-6600</v>
+        <v>-6966</v>
       </c>
       <c r="J89" s="7">
         <f>J79+J87</f>
-        <v>-7600</v>
+        <v>-8149</v>
       </c>
       <c r="K89" s="7">
         <f>K79+K87</f>
-        <v>-9600</v>
+        <v>-8332</v>
       </c>
       <c r="M89" s="2">
         <f>SUM(G89:K89)</f>
-        <v>-28400</v>
+        <v>-28230</v>
       </c>
       <c r="O89" s="2">
-        <f>M89-fyra_typfall_tid1!M89</f>
-        <v>-12860</v>
+        <f>M89-'fyra_typfall_tid1 (2)'!M89</f>
+        <v>-11092</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update index.html to specify the four groups (AA, BB, CC, DD) in the financial forecasting context, enhancing clarity in the presentation of group capabilities. The changes aim to improve user understanding of the different funding scenarios and their implications.
</commit_message>
<xml_diff>
--- a/ekonomikommunikation/260903/ekonomikommunikation.xlsx
+++ b/ekonomikommunikation/260903/ekonomikommunikation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ekonomi/ekonomikommunikation/260903/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="308" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C53F9C82-604B-4C3C-9636-1C63B095C42F}"/>
+  <xr:revisionPtr revIDLastSave="311" documentId="8_{9726B3CA-AB78-4A98-A934-370800F06452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47385CCB-4F4A-44F4-937E-42584095CFF6}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{639CD5D9-9986-427A-B3BB-8D4032026D07}"/>
   </bookViews>
   <sheets>
     <sheet name="fyra_typfall_tid1" sheetId="1" r:id="rId1"/>
@@ -2801,7 +2801,7 @@
         <v>5</v>
       </c>
       <c r="G34" s="2">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="G35" s="3">
         <f>SUM(G28:G34)</f>
-        <v>11300</v>
+        <v>10100</v>
       </c>
       <c r="H35" s="3">
         <f>SUM(H28:H34)</f>
@@ -2978,7 +2978,7 @@
       </c>
       <c r="G45" s="7">
         <f>G35+G43</f>
-        <v>1260</v>
+        <v>60</v>
       </c>
       <c r="H45" s="7">
         <f>H35+H43</f>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="M45" s="2">
         <f>SUM(G45:L45)</f>
-        <v>-3838</v>
+        <v>-5038</v>
       </c>
     </row>
     <row r="48" spans="6:13" x14ac:dyDescent="0.25">
@@ -3132,7 +3132,7 @@
         <v>5</v>
       </c>
       <c r="G56" s="2">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="G57" s="3">
         <f>SUM(G50:G56)</f>
-        <v>11300</v>
+        <v>10100</v>
       </c>
       <c r="H57" s="3">
         <f>SUM(H50:H56)</f>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="G67" s="2">
         <f>G57+G65</f>
-        <v>1260</v>
+        <v>60</v>
       </c>
       <c r="H67" s="2">
         <f>H57+H65</f>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="M67" s="2">
         <f>SUM(G67:L67)</f>
-        <v>-7438</v>
+        <v>-8638</v>
       </c>
     </row>
     <row r="70" spans="6:13" x14ac:dyDescent="0.25">
@@ -3446,7 +3446,7 @@
         <v>5</v>
       </c>
       <c r="G78" s="2">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
@@ -3459,7 +3459,7 @@
       </c>
       <c r="G79" s="3">
         <f>SUM(G72:G78)</f>
-        <v>11300</v>
+        <v>10100</v>
       </c>
       <c r="H79" s="3">
         <f>SUM(H72:H78)</f>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="G89" s="7">
         <f>G79+G87</f>
-        <v>1260</v>
+        <v>60</v>
       </c>
       <c r="H89" s="7">
         <f>H79+H87</f>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="M89" s="2">
         <f>SUM(G89:L89)</f>
-        <v>-17138</v>
+        <v>-18338</v>
       </c>
     </row>
   </sheetData>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="O45" s="2">
         <f>M45-'fyra_typfall_tid1 (2)'!M45</f>
-        <v>-5492</v>
+        <v>-4292</v>
       </c>
     </row>
     <row r="48" spans="6:15" x14ac:dyDescent="0.25">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="O67" s="2">
         <f>M67-'fyra_typfall_tid1 (2)'!M67</f>
-        <v>-8592</v>
+        <v>-7392</v>
       </c>
     </row>
     <row r="70" spans="6:15" x14ac:dyDescent="0.25">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="O89" s="2">
         <f>M89-'fyra_typfall_tid1 (2)'!M89</f>
-        <v>-11092</v>
+        <v>-9892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>